<commit_message>
file updates to fix for csv export
</commit_message>
<xml_diff>
--- a/InputData/fuels/FoVTStCT/Fraction of Vehicle Types Subject to Carbon Tax.xlsx
+++ b/InputData/fuels/FoVTStCT/Fraction of Vehicle Types Subject to Carbon Tax.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28906"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skorpius/My Drive/2024/FO local_EPS ICM/Diario/20250423_Last 50/OneDrive_3_30-04-2025/FoVTStCT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Mexico EPS\InputData\fuels\FoVTStCT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FFBA17-ED4F-1842-97AB-A59987879990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABDB4E6C-9F7C-4877-80A7-7248A1A166E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" firstSheet="1" activeTab="1" xr2:uid="{9AA6BDF2-7B91-4567-88A2-0D83F9E3E450}"/>
+    <workbookView xWindow="29760" yWindow="960" windowWidth="28800" windowHeight="14115" activeTab="1" xr2:uid="{9AA6BDF2-7B91-4567-88A2-0D83F9E3E450}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="BFoVTStCT" sheetId="3" r:id="rId2"/>
+    <sheet name="FoVTStCT" sheetId="3" r:id="rId2"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId3"/>
@@ -97,7 +97,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -348,9 +348,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -388,7 +388,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -494,7 +494,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -636,7 +636,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -645,32 +645,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE5FEEC-01CE-4291-999E-35B30A1256CF}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -687,14 +687,14 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AY28"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="1" max="1" width="46.33203125" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:51">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -849,7 +849,7 @@
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:51">
+    <row r="2" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:51">
+    <row r="3" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:51">
+    <row r="4" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:51">
+    <row r="5" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:51">
+    <row r="6" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:51">
+    <row r="7" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:51">
+    <row r="8" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -1811,7 +1811,7 @@
       <c r="AD8" s="4"/>
       <c r="AE8" s="4"/>
     </row>
-    <row r="9" spans="1:51">
+    <row r="9" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -1843,7 +1843,7 @@
       <c r="AD9" s="4"/>
       <c r="AE9" s="4"/>
     </row>
-    <row r="10" spans="1:51">
+    <row r="10" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -1875,7 +1875,7 @@
       <c r="AD10" s="4"/>
       <c r="AE10" s="4"/>
     </row>
-    <row r="11" spans="1:51">
+    <row r="11" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1907,7 +1907,7 @@
       <c r="AD11" s="4"/>
       <c r="AE11" s="4"/>
     </row>
-    <row r="12" spans="1:51">
+    <row r="12" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -1939,7 +1939,7 @@
       <c r="AD12" s="4"/>
       <c r="AE12" s="4"/>
     </row>
-    <row r="13" spans="1:51">
+    <row r="13" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -1971,7 +1971,7 @@
       <c r="AD13" s="4"/>
       <c r="AE13" s="4"/>
     </row>
-    <row r="14" spans="1:51">
+    <row r="14" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
@@ -2003,7 +2003,7 @@
       <c r="AD14" s="4"/>
       <c r="AE14" s="4"/>
     </row>
-    <row r="15" spans="1:51">
+    <row r="15" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -2035,7 +2035,7 @@
       <c r="AD15" s="4"/>
       <c r="AE15" s="4"/>
     </row>
-    <row r="16" spans="1:51">
+    <row r="16" spans="1:51" x14ac:dyDescent="0.3">
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -2067,7 +2067,7 @@
       <c r="AD16" s="4"/>
       <c r="AE16" s="4"/>
     </row>
-    <row r="17" spans="2:31">
+    <row r="17" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -2099,7 +2099,7 @@
       <c r="AD17" s="4"/>
       <c r="AE17" s="4"/>
     </row>
-    <row r="18" spans="2:31">
+    <row r="18" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
@@ -2131,7 +2131,7 @@
       <c r="AD18" s="4"/>
       <c r="AE18" s="4"/>
     </row>
-    <row r="19" spans="2:31">
+    <row r="19" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -2163,7 +2163,7 @@
       <c r="AD19" s="4"/>
       <c r="AE19" s="4"/>
     </row>
-    <row r="20" spans="2:31">
+    <row r="20" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
@@ -2195,7 +2195,7 @@
       <c r="AD20" s="4"/>
       <c r="AE20" s="4"/>
     </row>
-    <row r="21" spans="2:31">
+    <row r="21" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
@@ -2227,7 +2227,7 @@
       <c r="AD21" s="4"/>
       <c r="AE21" s="4"/>
     </row>
-    <row r="22" spans="2:31">
+    <row r="22" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
@@ -2259,7 +2259,7 @@
       <c r="AD22" s="4"/>
       <c r="AE22" s="4"/>
     </row>
-    <row r="23" spans="2:31">
+    <row r="23" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
@@ -2291,7 +2291,7 @@
       <c r="AD23" s="4"/>
       <c r="AE23" s="4"/>
     </row>
-    <row r="24" spans="2:31">
+    <row r="24" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
@@ -2323,7 +2323,7 @@
       <c r="AD24" s="4"/>
       <c r="AE24" s="4"/>
     </row>
-    <row r="25" spans="2:31">
+    <row r="25" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
@@ -2355,7 +2355,7 @@
       <c r="AD25" s="4"/>
       <c r="AE25" s="4"/>
     </row>
-    <row r="26" spans="2:31">
+    <row r="26" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -2387,7 +2387,7 @@
       <c r="AD26" s="4"/>
       <c r="AE26" s="4"/>
     </row>
-    <row r="28" spans="2:31">
+    <row r="28" spans="2:31" x14ac:dyDescent="0.3">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
@@ -2397,12 +2397,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -2546,6 +2540,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2556,13 +2556,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50494139-6273-4F48-B86A-62A19309365E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C08BB959-5157-48D1-8F2B-D1B25CDD486B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C08BB959-5157-48D1-8F2B-D1B25CDD486B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50494139-6273-4F48-B86A-62A19309365E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C866C1C1-CC33-4ADC-B8C6-022D2EBC063E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C866C1C1-CC33-4ADC-B8C6-022D2EBC063E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>